<commit_message>
added GPS to original columns in metadata files then re-ran data_processing file.
</commit_message>
<xml_diff>
--- a/data/Metadata18S_2017_2022_all.xlsx
+++ b/data/Metadata18S_2017_2022_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allisoncusick/Documents/Fjord_Phyto/FjordPhyto/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44C082F-9146-2047-AF7D-C94BC45D069B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193887AA-FC30-B947-8D3A-CBFB9DD7E362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13620" yWindow="500" windowWidth="20460" windowHeight="14900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8340" yWindow="500" windowWidth="20460" windowHeight="14900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
@@ -5513,8 +5513,12 @@
       <c r="K93" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="L93" s="15"/>
-      <c r="M93" s="15"/>
+      <c r="L93" s="15">
+        <v>-64.56</v>
+      </c>
+      <c r="M93" s="15">
+        <v>-62.426000000000002</v>
+      </c>
       <c r="N93" s="19" t="s">
         <v>349</v>
       </c>
@@ -5560,8 +5564,12 @@
       <c r="K94" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="L94" s="15"/>
-      <c r="M94" s="15"/>
+      <c r="L94" s="15">
+        <v>-64.56</v>
+      </c>
+      <c r="M94" s="15">
+        <v>-62.426000000000002</v>
+      </c>
       <c r="N94" s="19" t="s">
         <v>349</v>
       </c>

</xml_diff>